<commit_message>
Updated ITA_grids model - 2025-09-07 23:35
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{04EED4B9-BB26-4C1A-8E32-AB6B76D5E07B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{871DB88B-BD40-405C-98E5-2BD055C9A3D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7562,7 +7562,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09A3F36B-FF9E-4D84-BAB8-76661FFE2C92}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A132CB9-8805-4EB2-BD3C-0EDBD0651726}">
   <dimension ref="B9:D955"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -13373,10 +13373,10 @@
         <v>824</v>
       </c>
       <c r="C537">
-        <v>43.989961090000001</v>
+        <v>43.98996109117364</v>
       </c>
       <c r="D537">
-        <v>7.0498326220000003</v>
+        <v>7.049832621548787</v>
       </c>
     </row>
     <row r="538" spans="2:4">
@@ -13384,10 +13384,10 @@
         <v>825</v>
       </c>
       <c r="C538">
-        <v>44.439621270000004</v>
+        <v>44.439621273035918</v>
       </c>
       <c r="D538">
-        <v>7.0498326220000003</v>
+        <v>7.049832621548787</v>
       </c>
     </row>
     <row r="539" spans="2:4">
@@ -13395,10 +13395,10 @@
         <v>826</v>
       </c>
       <c r="C539">
-        <v>44.889281449999999</v>
+        <v>44.889281454898189</v>
       </c>
       <c r="D539">
-        <v>7.0498326220000003</v>
+        <v>7.049832621548787</v>
       </c>
     </row>
     <row r="540" spans="2:4">
@@ -13406,10 +13406,10 @@
         <v>827</v>
       </c>
       <c r="C540">
-        <v>45.338941640000002</v>
+        <v>45.338941636760453</v>
       </c>
       <c r="D540">
-        <v>7.0498326220000003</v>
+        <v>7.049832621548787</v>
       </c>
     </row>
     <row r="541" spans="2:4">
@@ -13417,10 +13417,10 @@
         <v>828</v>
       </c>
       <c r="C541">
-        <v>45.788601819999997</v>
+        <v>45.78860181862273</v>
       </c>
       <c r="D541">
-        <v>7.0498326220000003</v>
+        <v>7.049832621548787</v>
       </c>
     </row>
     <row r="542" spans="2:4">
@@ -13428,10 +13428,10 @@
         <v>829</v>
       </c>
       <c r="C542">
-        <v>43.989961090000001</v>
+        <v>43.98996109117364</v>
       </c>
       <c r="D542">
-        <v>7.6024493590000004</v>
+        <v>7.6024493593939084</v>
       </c>
     </row>
     <row r="543" spans="2:4">
@@ -13439,10 +13439,10 @@
         <v>830</v>
       </c>
       <c r="C543">
-        <v>44.439621270000004</v>
+        <v>44.439621273035918</v>
       </c>
       <c r="D543">
-        <v>7.6024493590000004</v>
+        <v>7.6024493593939084</v>
       </c>
     </row>
     <row r="544" spans="2:4">
@@ -13450,10 +13450,10 @@
         <v>831</v>
       </c>
       <c r="C544">
-        <v>44.889281449999999</v>
+        <v>44.889281454898189</v>
       </c>
       <c r="D544">
-        <v>7.6024493590000004</v>
+        <v>7.6024493593939084</v>
       </c>
     </row>
     <row r="545" spans="2:4">
@@ -13461,10 +13461,10 @@
         <v>832</v>
       </c>
       <c r="C545">
-        <v>45.338941640000002</v>
+        <v>45.338941636760453</v>
       </c>
       <c r="D545">
-        <v>7.6024493590000004</v>
+        <v>7.6024493593939084</v>
       </c>
     </row>
     <row r="546" spans="2:4">
@@ -13472,10 +13472,10 @@
         <v>833</v>
       </c>
       <c r="C546">
-        <v>45.788601819999997</v>
+        <v>45.78860181862273</v>
       </c>
       <c r="D546">
-        <v>7.6024493590000004</v>
+        <v>7.6024493593939084</v>
       </c>
     </row>
     <row r="547" spans="2:4">
@@ -13483,10 +13483,10 @@
         <v>834</v>
       </c>
       <c r="C547">
-        <v>39.043699089999997</v>
+        <v>39.043699090688669</v>
       </c>
       <c r="D547">
-        <v>8.1550660970000006</v>
+        <v>8.1550660972390308</v>
       </c>
     </row>
     <row r="548" spans="2:4">
@@ -13494,10 +13494,10 @@
         <v>835</v>
       </c>
       <c r="C548">
-        <v>39.493359269999999</v>
+        <v>39.493359272550933</v>
       </c>
       <c r="D548">
-        <v>8.1550660970000006</v>
+        <v>8.1550660972390308</v>
       </c>
     </row>
     <row r="549" spans="2:4">
@@ -13505,10 +13505,10 @@
         <v>836</v>
       </c>
       <c r="C549">
-        <v>39.943019450000001</v>
+        <v>39.943019454413211</v>
       </c>
       <c r="D549">
-        <v>8.1550660970000006</v>
+        <v>8.1550660972390308</v>
       </c>
     </row>
     <row r="550" spans="2:4">
@@ -13516,10 +13516,10 @@
         <v>837</v>
       </c>
       <c r="C550">
-        <v>40.392679639999997</v>
+        <v>40.392679636275481</v>
       </c>
       <c r="D550">
-        <v>8.1550660970000006</v>
+        <v>8.1550660972390308</v>
       </c>
     </row>
     <row r="551" spans="2:4">
@@ -13527,10 +13527,10 @@
         <v>838</v>
       </c>
       <c r="C551">
-        <v>40.842339819999999</v>
+        <v>40.842339818137752</v>
       </c>
       <c r="D551">
-        <v>8.1550660970000006</v>
+        <v>8.1550660972390308</v>
       </c>
     </row>
     <row r="552" spans="2:4">
@@ -13538,10 +13538,10 @@
         <v>839</v>
       </c>
       <c r="C552">
-        <v>41.292000000000002</v>
+        <v>41.292000000000023</v>
       </c>
       <c r="D552">
-        <v>8.1550660970000006</v>
+        <v>8.1550660972390308</v>
       </c>
     </row>
     <row r="553" spans="2:4">
@@ -13549,10 +13549,10 @@
         <v>840</v>
       </c>
       <c r="C553">
-        <v>43.989961090000001</v>
+        <v>43.98996109117364</v>
       </c>
       <c r="D553">
-        <v>8.1550660970000006</v>
+        <v>8.1550660972390308</v>
       </c>
     </row>
     <row r="554" spans="2:4">
@@ -13560,10 +13560,10 @@
         <v>841</v>
       </c>
       <c r="C554">
-        <v>44.439621270000004</v>
+        <v>44.439621273035918</v>
       </c>
       <c r="D554">
-        <v>8.1550660970000006</v>
+        <v>8.1550660972390308</v>
       </c>
     </row>
     <row r="555" spans="2:4">
@@ -13571,10 +13571,10 @@
         <v>842</v>
       </c>
       <c r="C555">
-        <v>44.889281449999999</v>
+        <v>44.889281454898189</v>
       </c>
       <c r="D555">
-        <v>8.1550660970000006</v>
+        <v>8.1550660972390308</v>
       </c>
     </row>
     <row r="556" spans="2:4">
@@ -13582,10 +13582,10 @@
         <v>843</v>
       </c>
       <c r="C556">
-        <v>45.338941640000002</v>
+        <v>45.338941636760453</v>
       </c>
       <c r="D556">
-        <v>8.1550660970000006</v>
+        <v>8.1550660972390308</v>
       </c>
     </row>
     <row r="557" spans="2:4">
@@ -13593,10 +13593,10 @@
         <v>844</v>
       </c>
       <c r="C557">
-        <v>45.788601819999997</v>
+        <v>45.78860181862273</v>
       </c>
       <c r="D557">
-        <v>8.1550660970000006</v>
+        <v>8.1550660972390308</v>
       </c>
     </row>
     <row r="558" spans="2:4">
@@ -13604,10 +13604,10 @@
         <v>845</v>
       </c>
       <c r="C558">
-        <v>46.238261999999999</v>
+        <v>46.238262000485001</v>
       </c>
       <c r="D558">
-        <v>8.1550660970000006</v>
+        <v>8.1550660972390308</v>
       </c>
     </row>
     <row r="559" spans="2:4">
@@ -13615,10 +13615,10 @@
         <v>846</v>
       </c>
       <c r="C559">
-        <v>39.043699089999997</v>
+        <v>39.043699090688662</v>
       </c>
       <c r="D559">
-        <v>8.707682835</v>
+        <v>8.7076828350841513</v>
       </c>
     </row>
     <row r="560" spans="2:4">
@@ -13626,10 +13626,10 @@
         <v>847</v>
       </c>
       <c r="C560">
-        <v>39.493359269999999</v>
+        <v>39.49335927255094</v>
       </c>
       <c r="D560">
-        <v>8.707682835</v>
+        <v>8.7076828350841513</v>
       </c>
     </row>
     <row r="561" spans="2:4">
@@ -13637,10 +13637,10 @@
         <v>848</v>
       </c>
       <c r="C561">
-        <v>39.943019450000001</v>
+        <v>39.943019454413196</v>
       </c>
       <c r="D561">
-        <v>8.707682835</v>
+        <v>8.7076828350841513</v>
       </c>
     </row>
     <row r="562" spans="2:4">
@@ -13648,10 +13648,10 @@
         <v>849</v>
       </c>
       <c r="C562">
-        <v>40.392679639999997</v>
+        <v>40.392679636275481</v>
       </c>
       <c r="D562">
-        <v>8.707682835</v>
+        <v>8.7076828350841513</v>
       </c>
     </row>
     <row r="563" spans="2:4">
@@ -13659,10 +13659,10 @@
         <v>850</v>
       </c>
       <c r="C563">
-        <v>40.842339819999999</v>
+        <v>40.842339818137752</v>
       </c>
       <c r="D563">
-        <v>8.707682835</v>
+        <v>8.7076828350841513</v>
       </c>
     </row>
     <row r="564" spans="2:4">
@@ -13670,10 +13670,10 @@
         <v>851</v>
       </c>
       <c r="C564">
-        <v>41.292000000000002</v>
+        <v>41.292000000000023</v>
       </c>
       <c r="D564">
-        <v>8.707682835</v>
+        <v>8.7076828350841513</v>
       </c>
     </row>
     <row r="565" spans="2:4">
@@ -13681,10 +13681,10 @@
         <v>852</v>
       </c>
       <c r="C565">
-        <v>44.439621270000004</v>
+        <v>44.439621273035918</v>
       </c>
       <c r="D565">
-        <v>8.707682835</v>
+        <v>8.7076828350841513</v>
       </c>
     </row>
     <row r="566" spans="2:4">
@@ -13692,10 +13692,10 @@
         <v>853</v>
       </c>
       <c r="C566">
-        <v>44.889281449999999</v>
+        <v>44.889281454898182</v>
       </c>
       <c r="D566">
-        <v>8.707682835</v>
+        <v>8.7076828350841513</v>
       </c>
     </row>
     <row r="567" spans="2:4">
@@ -13703,10 +13703,10 @@
         <v>854</v>
       </c>
       <c r="C567">
-        <v>45.338941640000002</v>
+        <v>45.338941636760453</v>
       </c>
       <c r="D567">
-        <v>8.707682835</v>
+        <v>8.7076828350841513</v>
       </c>
     </row>
     <row r="568" spans="2:4">
@@ -13714,10 +13714,10 @@
         <v>855</v>
       </c>
       <c r="C568">
-        <v>45.788601819999997</v>
+        <v>45.78860181862273</v>
       </c>
       <c r="D568">
-        <v>8.707682835</v>
+        <v>8.7076828350841513</v>
       </c>
     </row>
     <row r="569" spans="2:4">
@@ -13725,10 +13725,10 @@
         <v>856</v>
       </c>
       <c r="C569">
-        <v>46.238261999999999</v>
+        <v>46.238262000485001</v>
       </c>
       <c r="D569">
-        <v>8.707682835</v>
+        <v>8.7076828350841513</v>
       </c>
     </row>
     <row r="570" spans="2:4">
@@ -13736,10 +13736,10 @@
         <v>857</v>
       </c>
       <c r="C570">
-        <v>39.043699089999997</v>
+        <v>39.043699090688662</v>
       </c>
       <c r="D570">
-        <v>9.2602995729999993</v>
+        <v>9.2602995729292719</v>
       </c>
     </row>
     <row r="571" spans="2:4">
@@ -13747,10 +13747,10 @@
         <v>858</v>
       </c>
       <c r="C571">
-        <v>39.493359269999999</v>
+        <v>39.49335927255094</v>
       </c>
       <c r="D571">
-        <v>9.2602995729999993</v>
+        <v>9.2602995729292719</v>
       </c>
     </row>
     <row r="572" spans="2:4">
@@ -13758,10 +13758,10 @@
         <v>859</v>
       </c>
       <c r="C572">
-        <v>39.943019450000001</v>
+        <v>39.943019454413196</v>
       </c>
       <c r="D572">
-        <v>9.2602995729999993</v>
+        <v>9.2602995729292719</v>
       </c>
     </row>
     <row r="573" spans="2:4">
@@ -13769,10 +13769,10 @@
         <v>860</v>
       </c>
       <c r="C573">
-        <v>40.392679639999997</v>
+        <v>40.392679636275481</v>
       </c>
       <c r="D573">
-        <v>9.2602995729999993</v>
+        <v>9.2602995729292719</v>
       </c>
     </row>
     <row r="574" spans="2:4">
@@ -13780,10 +13780,10 @@
         <v>861</v>
       </c>
       <c r="C574">
-        <v>40.842339819999999</v>
+        <v>40.842339818137752</v>
       </c>
       <c r="D574">
-        <v>9.2602995729999993</v>
+        <v>9.2602995729292719</v>
       </c>
     </row>
     <row r="575" spans="2:4">
@@ -13791,10 +13791,10 @@
         <v>862</v>
       </c>
       <c r="C575">
-        <v>41.292000000000002</v>
+        <v>41.292000000000023</v>
       </c>
       <c r="D575">
-        <v>9.2602995729999993</v>
+        <v>9.2602995729292719</v>
       </c>
     </row>
     <row r="576" spans="2:4">
@@ -13802,10 +13802,10 @@
         <v>863</v>
       </c>
       <c r="C576">
-        <v>44.439621270000004</v>
+        <v>44.439621273035918</v>
       </c>
       <c r="D576">
-        <v>9.2602995729999993</v>
+        <v>9.2602995729292719</v>
       </c>
     </row>
     <row r="577" spans="2:4">
@@ -13813,10 +13813,10 @@
         <v>864</v>
       </c>
       <c r="C577">
-        <v>44.889281449999999</v>
+        <v>44.889281454898182</v>
       </c>
       <c r="D577">
-        <v>9.2602995729999993</v>
+        <v>9.2602995729292719</v>
       </c>
     </row>
     <row r="578" spans="2:4">
@@ -13824,10 +13824,10 @@
         <v>865</v>
       </c>
       <c r="C578">
-        <v>45.338941640000002</v>
+        <v>45.338941636760453</v>
       </c>
       <c r="D578">
-        <v>9.2602995729999993</v>
+        <v>9.2602995729292719</v>
       </c>
     </row>
     <row r="579" spans="2:4">
@@ -13835,10 +13835,10 @@
         <v>866</v>
       </c>
       <c r="C579">
-        <v>45.788601819999997</v>
+        <v>45.78860181862273</v>
       </c>
       <c r="D579">
-        <v>9.2602995729999993</v>
+        <v>9.2602995729292719</v>
       </c>
     </row>
     <row r="580" spans="2:4">
@@ -13846,10 +13846,10 @@
         <v>867</v>
       </c>
       <c r="C580">
-        <v>46.238261999999999</v>
+        <v>46.238262000485001</v>
       </c>
       <c r="D580">
-        <v>9.2602995729999993</v>
+        <v>9.2602995729292719</v>
       </c>
     </row>
     <row r="581" spans="2:4">
@@ -13857,10 +13857,10 @@
         <v>868</v>
       </c>
       <c r="C581">
-        <v>46.687922180000001</v>
+        <v>46.687922182347272</v>
       </c>
       <c r="D581">
-        <v>9.2602995729999993</v>
+        <v>9.2602995729292719</v>
       </c>
     </row>
     <row r="582" spans="2:4">
@@ -13868,10 +13868,10 @@
         <v>869</v>
       </c>
       <c r="C582">
-        <v>39.043699089999997</v>
+        <v>39.043699090688662</v>
       </c>
       <c r="D582">
-        <v>9.8129163110000004</v>
+        <v>9.8129163107743924</v>
       </c>
     </row>
     <row r="583" spans="2:4">
@@ -13879,10 +13879,10 @@
         <v>870</v>
       </c>
       <c r="C583">
-        <v>39.493359269999999</v>
+        <v>39.49335927255094</v>
       </c>
       <c r="D583">
-        <v>9.8129163110000004</v>
+        <v>9.8129163107743924</v>
       </c>
     </row>
     <row r="584" spans="2:4">
@@ -13890,10 +13890,10 @@
         <v>871</v>
       </c>
       <c r="C584">
-        <v>39.943019450000001</v>
+        <v>39.943019454413196</v>
       </c>
       <c r="D584">
-        <v>9.8129163110000004</v>
+        <v>9.8129163107743924</v>
       </c>
     </row>
     <row r="585" spans="2:4">
@@ -13901,10 +13901,10 @@
         <v>872</v>
       </c>
       <c r="C585">
-        <v>40.392679639999997</v>
+        <v>40.392679636275481</v>
       </c>
       <c r="D585">
-        <v>9.8129163110000004</v>
+        <v>9.8129163107743924</v>
       </c>
     </row>
     <row r="586" spans="2:4">
@@ -13912,10 +13912,10 @@
         <v>873</v>
       </c>
       <c r="C586">
-        <v>40.842339819999999</v>
+        <v>40.842339818137752</v>
       </c>
       <c r="D586">
-        <v>9.8129163110000004</v>
+        <v>9.8129163107743924</v>
       </c>
     </row>
     <row r="587" spans="2:4">
@@ -13923,10 +13923,10 @@
         <v>874</v>
       </c>
       <c r="C587">
-        <v>41.292000000000002</v>
+        <v>41.292000000000023</v>
       </c>
       <c r="D587">
-        <v>9.8129163110000004</v>
+        <v>9.8129163107743924</v>
       </c>
     </row>
     <row r="588" spans="2:4">
@@ -13934,10 +13934,10 @@
         <v>875</v>
       </c>
       <c r="C588">
-        <v>42.640980550000002</v>
+        <v>42.640980545586842</v>
       </c>
       <c r="D588">
-        <v>9.8129163110000004</v>
+        <v>9.8129163107743924</v>
       </c>
     </row>
     <row r="589" spans="2:4">
@@ -13945,10 +13945,10 @@
         <v>876</v>
       </c>
       <c r="C589">
-        <v>43.989961090000001</v>
+        <v>43.989961091173647</v>
       </c>
       <c r="D589">
-        <v>9.8129163110000004</v>
+        <v>9.8129163107743924</v>
       </c>
     </row>
     <row r="590" spans="2:4">
@@ -13956,10 +13956,10 @@
         <v>877</v>
       </c>
       <c r="C590">
-        <v>44.439621270000004</v>
+        <v>44.439621273035918</v>
       </c>
       <c r="D590">
-        <v>9.8129163110000004</v>
+        <v>9.8129163107743924</v>
       </c>
     </row>
     <row r="591" spans="2:4">
@@ -13967,10 +13967,10 @@
         <v>878</v>
       </c>
       <c r="C591">
-        <v>44.889281449999999</v>
+        <v>44.889281454898182</v>
       </c>
       <c r="D591">
-        <v>9.8129163110000004</v>
+        <v>9.8129163107743924</v>
       </c>
     </row>
     <row r="592" spans="2:4">
@@ -13978,10 +13978,10 @@
         <v>879</v>
       </c>
       <c r="C592">
-        <v>45.338941640000002</v>
+        <v>45.338941636760453</v>
       </c>
       <c r="D592">
-        <v>9.8129163110000004</v>
+        <v>9.8129163107743924</v>
       </c>
     </row>
     <row r="593" spans="2:4">
@@ -13989,10 +13989,10 @@
         <v>880</v>
       </c>
       <c r="C593">
-        <v>45.788601819999997</v>
+        <v>45.78860181862273</v>
       </c>
       <c r="D593">
-        <v>9.8129163110000004</v>
+        <v>9.8129163107743924</v>
       </c>
     </row>
     <row r="594" spans="2:4">
@@ -14000,10 +14000,10 @@
         <v>881</v>
       </c>
       <c r="C594">
-        <v>46.238261999999999</v>
+        <v>46.238262000485001</v>
       </c>
       <c r="D594">
-        <v>9.8129163110000004</v>
+        <v>9.8129163107743924</v>
       </c>
     </row>
     <row r="595" spans="2:4">
@@ -14011,10 +14011,10 @@
         <v>882</v>
       </c>
       <c r="C595">
-        <v>46.687922180000001</v>
+        <v>46.687922182347272</v>
       </c>
       <c r="D595">
-        <v>9.8129163110000004</v>
+        <v>9.8129163107743924</v>
       </c>
     </row>
     <row r="596" spans="2:4">
@@ -14022,10 +14022,10 @@
         <v>883</v>
       </c>
       <c r="C596">
-        <v>42.640980550000002</v>
+        <v>42.640980545586842</v>
       </c>
       <c r="D596">
-        <v>10.36553305</v>
+        <v>10.365533048619511</v>
       </c>
     </row>
     <row r="597" spans="2:4">
@@ -14033,10 +14033,10 @@
         <v>884</v>
       </c>
       <c r="C597">
-        <v>43.090640729999997</v>
+        <v>43.090640727449099</v>
       </c>
       <c r="D597">
-        <v>10.36553305</v>
+        <v>10.365533048619511</v>
       </c>
     </row>
     <row r="598" spans="2:4">
@@ -14044,10 +14044,10 @@
         <v>885</v>
       </c>
       <c r="C598">
-        <v>43.540300909999999</v>
+        <v>43.54030090931137</v>
       </c>
       <c r="D598">
-        <v>10.36553305</v>
+        <v>10.365533048619511</v>
       </c>
     </row>
     <row r="599" spans="2:4">
@@ -14055,10 +14055,10 @@
         <v>886</v>
       </c>
       <c r="C599">
-        <v>43.989961090000001</v>
+        <v>43.989961091173647</v>
       </c>
       <c r="D599">
-        <v>10.36553305</v>
+        <v>10.365533048619511</v>
       </c>
     </row>
     <row r="600" spans="2:4">
@@ -14066,10 +14066,10 @@
         <v>887</v>
       </c>
       <c r="C600">
-        <v>44.439621270000004</v>
+        <v>44.439621273035918</v>
       </c>
       <c r="D600">
-        <v>10.36553305</v>
+        <v>10.365533048619511</v>
       </c>
     </row>
     <row r="601" spans="2:4">
@@ -14077,10 +14077,10 @@
         <v>888</v>
       </c>
       <c r="C601">
-        <v>44.889281449999999</v>
+        <v>44.889281454898182</v>
       </c>
       <c r="D601">
-        <v>10.36553305</v>
+        <v>10.365533048619511</v>
       </c>
     </row>
     <row r="602" spans="2:4">
@@ -14088,10 +14088,10 @@
         <v>889</v>
       </c>
       <c r="C602">
-        <v>45.338941640000002</v>
+        <v>45.338941636760453</v>
       </c>
       <c r="D602">
-        <v>10.36553305</v>
+        <v>10.365533048619511</v>
       </c>
     </row>
     <row r="603" spans="2:4">
@@ -14099,10 +14099,10 @@
         <v>890</v>
       </c>
       <c r="C603">
-        <v>45.788601819999997</v>
+        <v>45.78860181862273</v>
       </c>
       <c r="D603">
-        <v>10.36553305</v>
+        <v>10.365533048619511</v>
       </c>
     </row>
     <row r="604" spans="2:4">
@@ -14110,10 +14110,10 @@
         <v>891</v>
       </c>
       <c r="C604">
-        <v>46.238261999999999</v>
+        <v>46.238262000485001</v>
       </c>
       <c r="D604">
-        <v>10.36553305</v>
+        <v>10.365533048619511</v>
       </c>
     </row>
     <row r="605" spans="2:4">
@@ -14121,10 +14121,10 @@
         <v>892</v>
       </c>
       <c r="C605">
-        <v>46.687922180000001</v>
+        <v>46.687922182347272</v>
       </c>
       <c r="D605">
-        <v>10.36553305</v>
+        <v>10.365533048619511</v>
       </c>
     </row>
     <row r="606" spans="2:4">
@@ -14132,10 +14132,10 @@
         <v>893</v>
       </c>
       <c r="C606">
-        <v>36.795398179999999</v>
+        <v>36.795398181377323</v>
       </c>
       <c r="D606">
-        <v>10.918149789999999</v>
+        <v>10.918149786464632</v>
       </c>
     </row>
     <row r="607" spans="2:4">
@@ -14143,10 +14143,10 @@
         <v>894</v>
       </c>
       <c r="C607">
-        <v>42.191320359999999</v>
+        <v>42.191320363724557</v>
       </c>
       <c r="D607">
-        <v>10.918149789999999</v>
+        <v>10.918149786464632</v>
       </c>
     </row>
     <row r="608" spans="2:4">
@@ -14154,10 +14154,10 @@
         <v>895</v>
       </c>
       <c r="C608">
-        <v>42.640980550000002</v>
+        <v>42.640980545586842</v>
       </c>
       <c r="D608">
-        <v>10.918149789999999</v>
+        <v>10.918149786464632</v>
       </c>
     </row>
     <row r="609" spans="2:4">
@@ -14165,10 +14165,10 @@
         <v>896</v>
       </c>
       <c r="C609">
-        <v>43.090640729999997</v>
+        <v>43.090640727449099</v>
       </c>
       <c r="D609">
-        <v>10.918149789999999</v>
+        <v>10.918149786464632</v>
       </c>
     </row>
     <row r="610" spans="2:4">
@@ -14176,10 +14176,10 @@
         <v>897</v>
       </c>
       <c r="C610">
-        <v>43.540300909999999</v>
+        <v>43.54030090931137</v>
       </c>
       <c r="D610">
-        <v>10.918149789999999</v>
+        <v>10.918149786464632</v>
       </c>
     </row>
     <row r="611" spans="2:4">
@@ -14187,10 +14187,10 @@
         <v>898</v>
       </c>
       <c r="C611">
-        <v>43.989961090000001</v>
+        <v>43.989961091173647</v>
       </c>
       <c r="D611">
-        <v>10.918149789999999</v>
+        <v>10.918149786464632</v>
       </c>
     </row>
     <row r="612" spans="2:4">
@@ -14198,10 +14198,10 @@
         <v>899</v>
       </c>
       <c r="C612">
-        <v>44.439621270000004</v>
+        <v>44.439621273035918</v>
       </c>
       <c r="D612">
-        <v>10.918149789999999</v>
+        <v>10.918149786464632</v>
       </c>
     </row>
     <row r="613" spans="2:4">
@@ -14209,10 +14209,10 @@
         <v>900</v>
       </c>
       <c r="C613">
-        <v>44.889281449999999</v>
+        <v>44.889281454898182</v>
       </c>
       <c r="D613">
-        <v>10.918149789999999</v>
+        <v>10.918149786464632</v>
       </c>
     </row>
     <row r="614" spans="2:4">
@@ -14220,10 +14220,10 @@
         <v>901</v>
       </c>
       <c r="C614">
-        <v>45.338941640000002</v>
+        <v>45.338941636760453</v>
       </c>
       <c r="D614">
-        <v>10.918149789999999</v>
+        <v>10.918149786464632</v>
       </c>
     </row>
     <row r="615" spans="2:4">
@@ -14231,10 +14231,10 @@
         <v>902</v>
       </c>
       <c r="C615">
-        <v>45.788601819999997</v>
+        <v>45.78860181862273</v>
       </c>
       <c r="D615">
-        <v>10.918149789999999</v>
+        <v>10.918149786464632</v>
       </c>
     </row>
     <row r="616" spans="2:4">
@@ -14242,10 +14242,10 @@
         <v>903</v>
       </c>
       <c r="C616">
-        <v>46.238261999999999</v>
+        <v>46.238262000485001</v>
       </c>
       <c r="D616">
-        <v>10.918149789999999</v>
+        <v>10.918149786464632</v>
       </c>
     </row>
     <row r="617" spans="2:4">
@@ -14253,10 +14253,10 @@
         <v>904</v>
       </c>
       <c r="C617">
-        <v>46.687922180000001</v>
+        <v>46.687922182347272</v>
       </c>
       <c r="D617">
-        <v>10.918149789999999</v>
+        <v>10.918149786464632</v>
       </c>
     </row>
     <row r="618" spans="2:4">
@@ -14264,10 +14264,10 @@
         <v>905</v>
       </c>
       <c r="C618">
-        <v>42.191320359999999</v>
+        <v>42.191320363724557</v>
       </c>
       <c r="D618">
-        <v>11.47076652</v>
+        <v>11.470766524309754</v>
       </c>
     </row>
     <row r="619" spans="2:4">
@@ -14275,10 +14275,10 @@
         <v>906</v>
       </c>
       <c r="C619">
-        <v>42.640980550000002</v>
+        <v>42.640980545586842</v>
       </c>
       <c r="D619">
-        <v>11.47076652</v>
+        <v>11.470766524309754</v>
       </c>
     </row>
     <row r="620" spans="2:4">
@@ -14286,10 +14286,10 @@
         <v>907</v>
       </c>
       <c r="C620">
-        <v>43.090640729999997</v>
+        <v>43.090640727449099</v>
       </c>
       <c r="D620">
-        <v>11.47076652</v>
+        <v>11.470766524309754</v>
       </c>
     </row>
     <row r="621" spans="2:4">
@@ -14297,10 +14297,10 @@
         <v>908</v>
       </c>
       <c r="C621">
-        <v>43.540300909999999</v>
+        <v>43.54030090931137</v>
       </c>
       <c r="D621">
-        <v>11.47076652</v>
+        <v>11.470766524309754</v>
       </c>
     </row>
     <row r="622" spans="2:4">
@@ -14308,10 +14308,10 @@
         <v>909</v>
       </c>
       <c r="C622">
-        <v>43.989961090000001</v>
+        <v>43.989961091173647</v>
       </c>
       <c r="D622">
-        <v>11.47076652</v>
+        <v>11.470766524309754</v>
       </c>
     </row>
     <row r="623" spans="2:4">
@@ -14319,10 +14319,10 @@
         <v>910</v>
       </c>
       <c r="C623">
-        <v>44.439621270000004</v>
+        <v>44.439621273035918</v>
       </c>
       <c r="D623">
-        <v>11.47076652</v>
+        <v>11.470766524309754</v>
       </c>
     </row>
     <row r="624" spans="2:4">
@@ -14330,10 +14330,10 @@
         <v>911</v>
       </c>
       <c r="C624">
-        <v>44.889281449999999</v>
+        <v>44.889281454898182</v>
       </c>
       <c r="D624">
-        <v>11.47076652</v>
+        <v>11.470766524309754</v>
       </c>
     </row>
     <row r="625" spans="2:4">
@@ -14341,10 +14341,10 @@
         <v>912</v>
       </c>
       <c r="C625">
-        <v>45.338941640000002</v>
+        <v>45.338941636760453</v>
       </c>
       <c r="D625">
-        <v>11.47076652</v>
+        <v>11.470766524309754</v>
       </c>
     </row>
     <row r="626" spans="2:4">
@@ -14352,10 +14352,10 @@
         <v>913</v>
       </c>
       <c r="C626">
-        <v>45.788601819999997</v>
+        <v>45.78860181862273</v>
       </c>
       <c r="D626">
-        <v>11.47076652</v>
+        <v>11.470766524309754</v>
       </c>
     </row>
     <row r="627" spans="2:4">
@@ -14363,10 +14363,10 @@
         <v>914</v>
       </c>
       <c r="C627">
-        <v>46.238261999999999</v>
+        <v>46.238262000485001</v>
       </c>
       <c r="D627">
-        <v>11.47076652</v>
+        <v>11.470766524309754</v>
       </c>
     </row>
     <row r="628" spans="2:4">
@@ -14374,10 +14374,10 @@
         <v>915</v>
       </c>
       <c r="C628">
-        <v>46.687922180000001</v>
+        <v>46.687922182347272</v>
       </c>
       <c r="D628">
-        <v>11.47076652</v>
+        <v>11.470766524309754</v>
       </c>
     </row>
     <row r="629" spans="2:4">
@@ -14385,10 +14385,10 @@
         <v>916</v>
       </c>
       <c r="C629">
-        <v>36.795398179999999</v>
+        <v>36.795398181377323</v>
       </c>
       <c r="D629">
-        <v>12.023383259999999</v>
+        <v>12.023383262154876</v>
       </c>
     </row>
     <row r="630" spans="2:4">
@@ -14396,10 +14396,10 @@
         <v>917</v>
       </c>
       <c r="C630">
-        <v>38.14437873</v>
+        <v>38.144378726964128</v>
       </c>
       <c r="D630">
-        <v>12.023383259999999</v>
+        <v>12.023383262154876</v>
       </c>
     </row>
     <row r="631" spans="2:4">
@@ -14407,10 +14407,10 @@
         <v>918</v>
       </c>
       <c r="C631">
-        <v>41.741660179999997</v>
+        <v>41.741660181862287</v>
       </c>
       <c r="D631">
-        <v>12.023383259999999</v>
+        <v>12.023383262154876</v>
       </c>
     </row>
     <row r="632" spans="2:4">
@@ -14418,10 +14418,10 @@
         <v>919</v>
       </c>
       <c r="C632">
-        <v>42.191320359999999</v>
+        <v>42.191320363724557</v>
       </c>
       <c r="D632">
-        <v>12.023383259999999</v>
+        <v>12.023383262154876</v>
       </c>
     </row>
     <row r="633" spans="2:4">
@@ -14429,10 +14429,10 @@
         <v>920</v>
       </c>
       <c r="C633">
-        <v>42.640980550000002</v>
+        <v>42.640980545586842</v>
       </c>
       <c r="D633">
-        <v>12.023383259999999</v>
+        <v>12.023383262154876</v>
       </c>
     </row>
     <row r="634" spans="2:4">
@@ -14440,10 +14440,10 @@
         <v>921</v>
       </c>
       <c r="C634">
-        <v>43.090640729999997</v>
+        <v>43.090640727449099</v>
       </c>
       <c r="D634">
-        <v>12.023383259999999</v>
+        <v>12.023383262154876</v>
       </c>
     </row>
     <row r="635" spans="2:4">
@@ -14451,10 +14451,10 @@
         <v>922</v>
       </c>
       <c r="C635">
-        <v>43.540300909999999</v>
+        <v>43.54030090931137</v>
       </c>
       <c r="D635">
-        <v>12.023383259999999</v>
+        <v>12.023383262154876</v>
       </c>
     </row>
     <row r="636" spans="2:4">
@@ -14462,10 +14462,10 @@
         <v>923</v>
       </c>
       <c r="C636">
-        <v>43.989961090000001</v>
+        <v>43.989961091173647</v>
       </c>
       <c r="D636">
-        <v>12.023383259999999</v>
+        <v>12.023383262154876</v>
       </c>
     </row>
     <row r="637" spans="2:4">
@@ -14473,10 +14473,10 @@
         <v>924</v>
       </c>
       <c r="C637">
-        <v>44.439621270000004</v>
+        <v>44.439621273035918</v>
       </c>
       <c r="D637">
-        <v>12.023383259999999</v>
+        <v>12.023383262154876</v>
       </c>
     </row>
     <row r="638" spans="2:4">
@@ -14484,10 +14484,10 @@
         <v>925</v>
       </c>
       <c r="C638">
-        <v>44.889281449999999</v>
+        <v>44.889281454898182</v>
       </c>
       <c r="D638">
-        <v>12.023383259999999</v>
+        <v>12.023383262154876</v>
       </c>
     </row>
     <row r="639" spans="2:4">
@@ -14495,10 +14495,10 @@
         <v>926</v>
       </c>
       <c r="C639">
-        <v>45.338941640000002</v>
+        <v>45.338941636760453</v>
       </c>
       <c r="D639">
-        <v>12.023383259999999</v>
+        <v>12.023383262154876</v>
       </c>
     </row>
     <row r="640" spans="2:4">
@@ -14506,10 +14506,10 @@
         <v>927</v>
       </c>
       <c r="C640">
-        <v>45.788601819999997</v>
+        <v>45.78860181862273</v>
       </c>
       <c r="D640">
-        <v>12.023383259999999</v>
+        <v>12.023383262154876</v>
       </c>
     </row>
     <row r="641" spans="2:4">
@@ -14517,10 +14517,10 @@
         <v>928</v>
       </c>
       <c r="C641">
-        <v>46.238261999999999</v>
+        <v>46.238262000485001</v>
       </c>
       <c r="D641">
-        <v>12.023383259999999</v>
+        <v>12.023383262154876</v>
       </c>
     </row>
     <row r="642" spans="2:4">
@@ -14528,10 +14528,10 @@
         <v>929</v>
       </c>
       <c r="C642">
-        <v>46.687922180000001</v>
+        <v>46.687922182347272</v>
       </c>
       <c r="D642">
-        <v>12.023383259999999</v>
+        <v>12.023383262154876</v>
       </c>
     </row>
     <row r="643" spans="2:4">
@@ -14539,10 +14539,10 @@
         <v>930</v>
       </c>
       <c r="C643">
-        <v>37.694718549999997</v>
+        <v>37.69471854510185</v>
       </c>
       <c r="D643">
-        <v>12.576000000000001</v>
+        <v>12.575999999999992</v>
       </c>
     </row>
     <row r="644" spans="2:4">
@@ -14550,10 +14550,10 @@
         <v>931</v>
       </c>
       <c r="C644">
-        <v>38.14437873</v>
+        <v>38.144378726964128</v>
       </c>
       <c r="D644">
-        <v>12.576000000000001</v>
+        <v>12.575999999999992</v>
       </c>
     </row>
     <row r="645" spans="2:4">
@@ -14561,10 +14561,10 @@
         <v>932</v>
       </c>
       <c r="C645">
-        <v>41.292000000000002</v>
+        <v>41.292000000000023</v>
       </c>
       <c r="D645">
-        <v>12.576000000000001</v>
+        <v>12.575999999999992</v>
       </c>
     </row>
     <row r="646" spans="2:4">
@@ -14572,10 +14572,10 @@
         <v>933</v>
       </c>
       <c r="C646">
-        <v>41.741660179999997</v>
+        <v>41.741660181862287</v>
       </c>
       <c r="D646">
-        <v>12.576000000000001</v>
+        <v>12.575999999999992</v>
       </c>
     </row>
     <row r="647" spans="2:4">
@@ -14583,10 +14583,10 @@
         <v>934</v>
       </c>
       <c r="C647">
-        <v>42.191320359999999</v>
+        <v>42.191320363724557</v>
       </c>
       <c r="D647">
-        <v>12.576000000000001</v>
+        <v>12.575999999999992</v>
       </c>
     </row>
     <row r="648" spans="2:4">
@@ -14594,10 +14594,10 @@
         <v>935</v>
       </c>
       <c r="C648">
-        <v>42.640980550000002</v>
+        <v>42.640980545586842</v>
       </c>
       <c r="D648">
-        <v>12.576000000000001</v>
+        <v>12.575999999999992</v>
       </c>
     </row>
     <row r="649" spans="2:4">
@@ -14605,10 +14605,10 @@
         <v>936</v>
       </c>
       <c r="C649">
-        <v>43.090640729999997</v>
+        <v>43.090640727449099</v>
       </c>
       <c r="D649">
-        <v>12.576000000000001</v>
+        <v>12.575999999999992</v>
       </c>
     </row>
     <row r="650" spans="2:4">
@@ -14616,10 +14616,10 @@
         <v>937</v>
       </c>
       <c r="C650">
-        <v>43.540300909999999</v>
+        <v>43.54030090931137</v>
       </c>
       <c r="D650">
-        <v>12.576000000000001</v>
+        <v>12.575999999999992</v>
       </c>
     </row>
     <row r="651" spans="2:4">
@@ -14627,10 +14627,10 @@
         <v>938</v>
       </c>
       <c r="C651">
-        <v>43.989961090000001</v>
+        <v>43.989961091173647</v>
       </c>
       <c r="D651">
-        <v>12.576000000000001</v>
+        <v>12.575999999999992</v>
       </c>
     </row>
     <row r="652" spans="2:4">
@@ -14638,10 +14638,10 @@
         <v>939</v>
       </c>
       <c r="C652">
-        <v>44.439621270000004</v>
+        <v>44.439621273035918</v>
       </c>
       <c r="D652">
-        <v>12.576000000000001</v>
+        <v>12.575999999999992</v>
       </c>
     </row>
     <row r="653" spans="2:4">
@@ -14649,10 +14649,10 @@
         <v>940</v>
       </c>
       <c r="C653">
-        <v>44.889281449999999</v>
+        <v>44.889281454898182</v>
       </c>
       <c r="D653">
-        <v>12.576000000000001</v>
+        <v>12.575999999999992</v>
       </c>
     </row>
     <row r="654" spans="2:4">
@@ -14660,10 +14660,10 @@
         <v>941</v>
       </c>
       <c r="C654">
-        <v>45.338941640000002</v>
+        <v>45.338941636760453</v>
       </c>
       <c r="D654">
-        <v>12.576000000000001</v>
+        <v>12.575999999999992</v>
       </c>
     </row>
     <row r="655" spans="2:4">
@@ -14671,10 +14671,10 @@
         <v>942</v>
       </c>
       <c r="C655">
-        <v>45.788601819999997</v>
+        <v>45.78860181862273</v>
       </c>
       <c r="D655">
-        <v>12.576000000000001</v>
+        <v>12.575999999999992</v>
       </c>
     </row>
     <row r="656" spans="2:4">
@@ -14682,10 +14682,10 @@
         <v>943</v>
       </c>
       <c r="C656">
-        <v>46.238261999999999</v>
+        <v>46.238262000485001</v>
       </c>
       <c r="D656">
-        <v>12.576000000000001</v>
+        <v>12.575999999999992</v>
       </c>
     </row>
     <row r="657" spans="2:4">
@@ -14693,10 +14693,10 @@
         <v>944</v>
       </c>
       <c r="C657">
-        <v>46.687922180000001</v>
+        <v>46.687922182347272</v>
       </c>
       <c r="D657">
-        <v>12.576000000000001</v>
+        <v>12.575999999999992</v>
       </c>
     </row>
     <row r="658" spans="2:4">
@@ -14704,10 +14704,10 @@
         <v>945</v>
       </c>
       <c r="C658">
-        <v>35.896077820000002</v>
+        <v>35.896077817652767</v>
       </c>
       <c r="D658">
-        <v>13.12861674</v>
+        <v>13.128616737845118</v>
       </c>
     </row>
     <row r="659" spans="2:4">
@@ -14715,10 +14715,10 @@
         <v>946</v>
       </c>
       <c r="C659">
-        <v>37.245058360000002</v>
+        <v>37.245058363239593</v>
       </c>
       <c r="D659">
-        <v>13.12861674</v>
+        <v>13.128616737845118</v>
       </c>
     </row>
     <row r="660" spans="2:4">
@@ -14726,10 +14726,10 @@
         <v>947</v>
       </c>
       <c r="C660">
-        <v>37.694718549999997</v>
+        <v>37.69471854510185</v>
       </c>
       <c r="D660">
-        <v>13.12861674</v>
+        <v>13.128616737845118</v>
       </c>
     </row>
     <row r="661" spans="2:4">
@@ -14737,10 +14737,10 @@
         <v>948</v>
       </c>
       <c r="C661">
-        <v>38.14437873</v>
+        <v>38.144378726964128</v>
       </c>
       <c r="D661">
-        <v>13.12861674</v>
+        <v>13.128616737845118</v>
       </c>
     </row>
     <row r="662" spans="2:4">
@@ -14748,10 +14748,10 @@
         <v>949</v>
       </c>
       <c r="C662">
-        <v>40.842339819999999</v>
+        <v>40.842339818137752</v>
       </c>
       <c r="D662">
-        <v>13.12861674</v>
+        <v>13.128616737845118</v>
       </c>
     </row>
     <row r="663" spans="2:4">
@@ -14759,10 +14759,10 @@
         <v>950</v>
       </c>
       <c r="C663">
-        <v>41.292000000000002</v>
+        <v>41.292000000000023</v>
       </c>
       <c r="D663">
-        <v>13.12861674</v>
+        <v>13.128616737845118</v>
       </c>
     </row>
     <row r="664" spans="2:4">
@@ -14770,10 +14770,10 @@
         <v>951</v>
       </c>
       <c r="C664">
-        <v>41.741660179999997</v>
+        <v>41.741660181862287</v>
       </c>
       <c r="D664">
-        <v>13.12861674</v>
+        <v>13.128616737845118</v>
       </c>
     </row>
     <row r="665" spans="2:4">
@@ -14781,10 +14781,10 @@
         <v>952</v>
       </c>
       <c r="C665">
-        <v>42.191320359999999</v>
+        <v>42.191320363724557</v>
       </c>
       <c r="D665">
-        <v>13.12861674</v>
+        <v>13.128616737845118</v>
       </c>
     </row>
     <row r="666" spans="2:4">
@@ -14792,10 +14792,10 @@
         <v>953</v>
       </c>
       <c r="C666">
-        <v>42.640980550000002</v>
+        <v>42.640980545586842</v>
       </c>
       <c r="D666">
-        <v>13.12861674</v>
+        <v>13.128616737845118</v>
       </c>
     </row>
     <row r="667" spans="2:4">
@@ -14803,10 +14803,10 @@
         <v>954</v>
       </c>
       <c r="C667">
-        <v>43.090640729999997</v>
+        <v>43.090640727449099</v>
       </c>
       <c r="D667">
-        <v>13.12861674</v>
+        <v>13.128616737845118</v>
       </c>
     </row>
     <row r="668" spans="2:4">
@@ -14814,10 +14814,10 @@
         <v>955</v>
       </c>
       <c r="C668">
-        <v>43.540300909999999</v>
+        <v>43.54030090931137</v>
       </c>
       <c r="D668">
-        <v>13.12861674</v>
+        <v>13.128616737845118</v>
       </c>
     </row>
     <row r="669" spans="2:4">
@@ -14825,10 +14825,10 @@
         <v>956</v>
       </c>
       <c r="C669">
-        <v>43.989961090000001</v>
+        <v>43.989961091173647</v>
       </c>
       <c r="D669">
-        <v>13.12861674</v>
+        <v>13.128616737845118</v>
       </c>
     </row>
     <row r="670" spans="2:4">
@@ -14836,10 +14836,10 @@
         <v>957</v>
       </c>
       <c r="C670">
-        <v>45.788601819999997</v>
+        <v>45.78860181862273</v>
       </c>
       <c r="D670">
-        <v>13.12861674</v>
+        <v>13.128616737845118</v>
       </c>
     </row>
     <row r="671" spans="2:4">
@@ -14847,10 +14847,10 @@
         <v>958</v>
       </c>
       <c r="C671">
-        <v>46.238261999999999</v>
+        <v>46.238262000485001</v>
       </c>
       <c r="D671">
-        <v>13.12861674</v>
+        <v>13.128616737845118</v>
       </c>
     </row>
     <row r="672" spans="2:4">
@@ -14858,10 +14858,10 @@
         <v>959</v>
       </c>
       <c r="C672">
-        <v>46.687922180000001</v>
+        <v>46.687922182347272</v>
       </c>
       <c r="D672">
-        <v>13.12861674</v>
+        <v>13.128616737845118</v>
       </c>
     </row>
     <row r="673" spans="2:4">
@@ -14869,10 +14869,10 @@
         <v>960</v>
       </c>
       <c r="C673">
-        <v>37.245058360000002</v>
+        <v>37.245058363239593</v>
       </c>
       <c r="D673">
-        <v>13.68123348</v>
+        <v>13.681233475690236</v>
       </c>
     </row>
     <row r="674" spans="2:4">
@@ -14880,10 +14880,10 @@
         <v>961</v>
       </c>
       <c r="C674">
-        <v>37.694718549999997</v>
+        <v>37.69471854510185</v>
       </c>
       <c r="D674">
-        <v>13.68123348</v>
+        <v>13.681233475690236</v>
       </c>
     </row>
     <row r="675" spans="2:4">
@@ -14891,10 +14891,10 @@
         <v>962</v>
       </c>
       <c r="C675">
-        <v>38.14437873</v>
+        <v>38.144378726964128</v>
       </c>
       <c r="D675">
-        <v>13.68123348</v>
+        <v>13.681233475690236</v>
       </c>
     </row>
     <row r="676" spans="2:4">
@@ -14902,10 +14902,10 @@
         <v>963</v>
       </c>
       <c r="C676">
-        <v>40.842339819999999</v>
+        <v>40.842339818137752</v>
       </c>
       <c r="D676">
-        <v>13.68123348</v>
+        <v>13.681233475690236</v>
       </c>
     </row>
     <row r="677" spans="2:4">
@@ -14913,10 +14913,10 @@
         <v>964</v>
       </c>
       <c r="C677">
-        <v>41.292000000000002</v>
+        <v>41.292000000000023</v>
       </c>
       <c r="D677">
-        <v>13.68123348</v>
+        <v>13.681233475690236</v>
       </c>
     </row>
     <row r="678" spans="2:4">
@@ -14924,10 +14924,10 @@
         <v>965</v>
       </c>
       <c r="C678">
-        <v>41.741660179999997</v>
+        <v>41.741660181862287</v>
       </c>
       <c r="D678">
-        <v>13.68123348</v>
+        <v>13.681233475690236</v>
       </c>
     </row>
     <row r="679" spans="2:4">
@@ -14935,10 +14935,10 @@
         <v>966</v>
       </c>
       <c r="C679">
-        <v>42.191320359999999</v>
+        <v>42.191320363724557</v>
       </c>
       <c r="D679">
-        <v>13.68123348</v>
+        <v>13.681233475690236</v>
       </c>
     </row>
     <row r="680" spans="2:4">
@@ -14946,10 +14946,10 @@
         <v>967</v>
       </c>
       <c r="C680">
-        <v>42.640980550000002</v>
+        <v>42.640980545586842</v>
       </c>
       <c r="D680">
-        <v>13.68123348</v>
+        <v>13.681233475690236</v>
       </c>
     </row>
     <row r="681" spans="2:4">
@@ -14957,10 +14957,10 @@
         <v>968</v>
       </c>
       <c r="C681">
-        <v>43.090640729999997</v>
+        <v>43.090640727449099</v>
       </c>
       <c r="D681">
-        <v>13.68123348</v>
+        <v>13.681233475690236</v>
       </c>
     </row>
     <row r="682" spans="2:4">
@@ -14968,10 +14968,10 @@
         <v>969</v>
       </c>
       <c r="C682">
-        <v>43.540300909999999</v>
+        <v>43.54030090931137</v>
       </c>
       <c r="D682">
-        <v>13.68123348</v>
+        <v>13.681233475690236</v>
       </c>
     </row>
     <row r="683" spans="2:4">
@@ -14979,10 +14979,10 @@
         <v>970</v>
       </c>
       <c r="C683">
-        <v>45.788601819999997</v>
+        <v>45.78860181862273</v>
       </c>
       <c r="D683">
-        <v>13.68123348</v>
+        <v>13.681233475690236</v>
       </c>
     </row>
     <row r="684" spans="2:4">
@@ -14990,10 +14990,10 @@
         <v>971</v>
       </c>
       <c r="C684">
-        <v>46.238261999999999</v>
+        <v>46.238262000485001</v>
       </c>
       <c r="D684">
-        <v>13.68123348</v>
+        <v>13.681233475690236</v>
       </c>
     </row>
     <row r="685" spans="2:4">
@@ -15001,10 +15001,10 @@
         <v>972</v>
       </c>
       <c r="C685">
-        <v>46.687922180000001</v>
+        <v>46.687922182347272</v>
       </c>
       <c r="D685">
-        <v>13.68123348</v>
+        <v>13.681233475690236</v>
       </c>
     </row>
     <row r="686" spans="2:4">
@@ -15012,10 +15012,10 @@
         <v>973</v>
       </c>
       <c r="C686">
-        <v>36.795398179999999</v>
+        <v>36.795398181377323</v>
       </c>
       <c r="D686">
-        <v>14.23385021</v>
+        <v>14.233850213535357</v>
       </c>
     </row>
     <row r="687" spans="2:4">
@@ -15023,10 +15023,10 @@
         <v>974</v>
       </c>
       <c r="C687">
-        <v>37.245058360000002</v>
+        <v>37.245058363239593</v>
       </c>
       <c r="D687">
-        <v>14.23385021</v>
+        <v>14.233850213535357</v>
       </c>
     </row>
     <row r="688" spans="2:4">
@@ -15034,10 +15034,10 @@
         <v>975</v>
       </c>
       <c r="C688">
-        <v>37.694718549999997</v>
+        <v>37.69471854510185</v>
       </c>
       <c r="D688">
-        <v>14.23385021</v>
+        <v>14.233850213535357</v>
       </c>
     </row>
     <row r="689" spans="2:4">
@@ -15045,10 +15045,10 @@
         <v>976</v>
       </c>
       <c r="C689">
-        <v>38.14437873</v>
+        <v>38.144378726964128</v>
       </c>
       <c r="D689">
-        <v>14.23385021</v>
+        <v>14.233850213535357</v>
       </c>
     </row>
     <row r="690" spans="2:4">
@@ -15056,10 +15056,10 @@
         <v>977</v>
       </c>
       <c r="C690">
-        <v>40.392679639999997</v>
+        <v>40.392679636275481</v>
       </c>
       <c r="D690">
-        <v>14.23385021</v>
+        <v>14.233850213535357</v>
       </c>
     </row>
     <row r="691" spans="2:4">
@@ -15067,10 +15067,10 @@
         <v>978</v>
       </c>
       <c r="C691">
-        <v>40.842339819999999</v>
+        <v>40.842339818137752</v>
       </c>
       <c r="D691">
-        <v>14.23385021</v>
+        <v>14.233850213535357</v>
       </c>
     </row>
     <row r="692" spans="2:4">
@@ -15078,10 +15078,10 @@
         <v>979</v>
       </c>
       <c r="C692">
-        <v>41.292000000000002</v>
+        <v>41.292000000000023</v>
       </c>
       <c r="D692">
-        <v>14.23385021</v>
+        <v>14.233850213535357</v>
       </c>
     </row>
     <row r="693" spans="2:4">
@@ -15089,10 +15089,10 @@
         <v>980</v>
       </c>
       <c r="C693">
-        <v>41.741660179999997</v>
+        <v>41.741660181862287</v>
       </c>
       <c r="D693">
-        <v>14.23385021</v>
+        <v>14.233850213535357</v>
       </c>
     </row>
     <row r="694" spans="2:4">
@@ -15100,10 +15100,10 @@
         <v>981</v>
       </c>
       <c r="C694">
-        <v>42.191320359999999</v>
+        <v>42.191320363724557</v>
       </c>
       <c r="D694">
-        <v>14.23385021</v>
+        <v>14.233850213535357</v>
       </c>
     </row>
     <row r="695" spans="2:4">
@@ -15111,10 +15111,10 @@
         <v>982</v>
       </c>
       <c r="C695">
-        <v>42.640980550000002</v>
+        <v>42.640980545586842</v>
       </c>
       <c r="D695">
-        <v>14.23385021</v>
+        <v>14.233850213535357</v>
       </c>
     </row>
     <row r="696" spans="2:4">
@@ -15122,10 +15122,10 @@
         <v>983</v>
       </c>
       <c r="C696">
-        <v>36.795398179999999</v>
+        <v>36.795398181377323</v>
       </c>
       <c r="D696">
-        <v>14.786466949999999</v>
+        <v>14.786466951380476</v>
       </c>
     </row>
     <row r="697" spans="2:4">
@@ -15133,10 +15133,10 @@
         <v>984</v>
       </c>
       <c r="C697">
-        <v>37.245058360000002</v>
+        <v>37.245058363239593</v>
       </c>
       <c r="D697">
-        <v>14.786466949999999</v>
+        <v>14.786466951380476</v>
       </c>
     </row>
     <row r="698" spans="2:4">
@@ -15144,10 +15144,10 @@
         <v>985</v>
       </c>
       <c r="C698">
-        <v>37.694718549999997</v>
+        <v>37.69471854510185</v>
       </c>
       <c r="D698">
-        <v>14.786466949999999</v>
+        <v>14.786466951380476</v>
       </c>
     </row>
     <row r="699" spans="2:4">
@@ -15155,10 +15155,10 @@
         <v>986</v>
       </c>
       <c r="C699">
-        <v>38.14437873</v>
+        <v>38.144378726964128</v>
       </c>
       <c r="D699">
-        <v>14.786466949999999</v>
+        <v>14.786466951380476</v>
       </c>
     </row>
     <row r="700" spans="2:4">
@@ -15166,10 +15166,10 @@
         <v>987</v>
       </c>
       <c r="C700">
-        <v>38.594038910000002</v>
+        <v>38.594038908826398</v>
       </c>
       <c r="D700">
-        <v>14.786466949999999</v>
+        <v>14.786466951380476</v>
       </c>
     </row>
     <row r="701" spans="2:4">
@@ -15177,10 +15177,10 @@
         <v>988</v>
       </c>
       <c r="C701">
-        <v>40.392679639999997</v>
+        <v>40.392679636275481</v>
       </c>
       <c r="D701">
-        <v>14.786466949999999</v>
+        <v>14.786466951380476</v>
       </c>
     </row>
     <row r="702" spans="2:4">
@@ -15188,10 +15188,10 @@
         <v>989</v>
       </c>
       <c r="C702">
-        <v>40.842339819999999</v>
+        <v>40.842339818137752</v>
       </c>
       <c r="D702">
-        <v>14.786466949999999</v>
+        <v>14.786466951380476</v>
       </c>
     </row>
     <row r="703" spans="2:4">
@@ -15199,10 +15199,10 @@
         <v>990</v>
       </c>
       <c r="C703">
-        <v>41.292000000000002</v>
+        <v>41.292000000000023</v>
       </c>
       <c r="D703">
-        <v>14.786466949999999</v>
+        <v>14.786466951380476</v>
       </c>
     </row>
     <row r="704" spans="2:4">
@@ -15210,10 +15210,10 @@
         <v>991</v>
       </c>
       <c r="C704">
-        <v>41.741660179999997</v>
+        <v>41.741660181862287</v>
       </c>
       <c r="D704">
-        <v>14.786466949999999</v>
+        <v>14.786466951380476</v>
       </c>
     </row>
     <row r="705" spans="2:4">
@@ -15221,10 +15221,10 @@
         <v>992</v>
       </c>
       <c r="C705">
-        <v>42.191320359999999</v>
+        <v>42.191320363724557</v>
       </c>
       <c r="D705">
-        <v>14.786466949999999</v>
+        <v>14.786466951380476</v>
       </c>
     </row>
     <row r="706" spans="2:4">
@@ -15232,10 +15232,10 @@
         <v>993</v>
       </c>
       <c r="C706">
-        <v>36.795398179999999</v>
+        <v>36.795398181377323</v>
       </c>
       <c r="D706">
-        <v>15.339083690000001</v>
+        <v>15.339083689225598</v>
       </c>
     </row>
     <row r="707" spans="2:4">
@@ -15243,10 +15243,10 @@
         <v>994</v>
       </c>
       <c r="C707">
-        <v>37.245058360000002</v>
+        <v>37.245058363239593</v>
       </c>
       <c r="D707">
-        <v>15.339083690000001</v>
+        <v>15.339083689225598</v>
       </c>
     </row>
     <row r="708" spans="2:4">
@@ -15254,10 +15254,10 @@
         <v>995</v>
       </c>
       <c r="C708">
-        <v>37.694718549999997</v>
+        <v>37.69471854510185</v>
       </c>
       <c r="D708">
-        <v>15.339083690000001</v>
+        <v>15.339083689225598</v>
       </c>
     </row>
     <row r="709" spans="2:4">
@@ -15265,10 +15265,10 @@
         <v>996</v>
       </c>
       <c r="C709">
-        <v>38.14437873</v>
+        <v>38.144378726964128</v>
       </c>
       <c r="D709">
-        <v>15.339083690000001</v>
+        <v>15.339083689225598</v>
       </c>
     </row>
     <row r="710" spans="2:4">
@@ -15276,10 +15276,10 @@
         <v>997</v>
       </c>
       <c r="C710">
-        <v>39.943019450000001</v>
+        <v>39.943019454413196</v>
       </c>
       <c r="D710">
-        <v>15.339083690000001</v>
+        <v>15.339083689225598</v>
       </c>
     </row>
     <row r="711" spans="2:4">
@@ -15287,10 +15287,10 @@
         <v>998</v>
       </c>
       <c r="C711">
-        <v>40.392679639999997</v>
+        <v>40.392679636275481</v>
       </c>
       <c r="D711">
-        <v>15.339083690000001</v>
+        <v>15.339083689225598</v>
       </c>
     </row>
     <row r="712" spans="2:4">
@@ -15298,10 +15298,10 @@
         <v>999</v>
       </c>
       <c r="C712">
-        <v>40.842339819999999</v>
+        <v>40.842339818137752</v>
       </c>
       <c r="D712">
-        <v>15.339083690000001</v>
+        <v>15.339083689225598</v>
       </c>
     </row>
     <row r="713" spans="2:4">
@@ -15309,10 +15309,10 @@
         <v>1000</v>
       </c>
       <c r="C713">
-        <v>41.292000000000002</v>
+        <v>41.292000000000023</v>
       </c>
       <c r="D713">
-        <v>15.339083690000001</v>
+        <v>15.339083689225598</v>
       </c>
     </row>
     <row r="714" spans="2:4">
@@ -15320,10 +15320,10 @@
         <v>1001</v>
       </c>
       <c r="C714">
-        <v>41.741660179999997</v>
+        <v>41.741660181862287</v>
       </c>
       <c r="D714">
-        <v>15.339083690000001</v>
+        <v>15.339083689225598</v>
       </c>
     </row>
     <row r="715" spans="2:4">
@@ -15331,10 +15331,10 @@
         <v>1002</v>
       </c>
       <c r="C715">
-        <v>42.191320359999999</v>
+        <v>42.191320363724557</v>
       </c>
       <c r="D715">
-        <v>15.339083690000001</v>
+        <v>15.339083689225598</v>
       </c>
     </row>
     <row r="716" spans="2:4">
@@ -15342,10 +15342,10 @@
         <v>1003</v>
       </c>
       <c r="C716">
-        <v>38.14437873</v>
+        <v>38.144378726964128</v>
       </c>
       <c r="D716">
-        <v>15.89170043</v>
+        <v>15.89170042707072</v>
       </c>
     </row>
     <row r="717" spans="2:4">
@@ -15353,10 +15353,10 @@
         <v>1004</v>
       </c>
       <c r="C717">
-        <v>38.594038910000002</v>
+        <v>38.594038908826391</v>
       </c>
       <c r="D717">
-        <v>15.89170043</v>
+        <v>15.89170042707072</v>
       </c>
     </row>
     <row r="718" spans="2:4">
@@ -15364,10 +15364,10 @@
         <v>1005</v>
       </c>
       <c r="C718">
-        <v>39.043699089999997</v>
+        <v>39.043699090688662</v>
       </c>
       <c r="D718">
-        <v>15.89170043</v>
+        <v>15.89170042707072</v>
       </c>
     </row>
     <row r="719" spans="2:4">
@@ -15375,10 +15375,10 @@
         <v>1006</v>
       </c>
       <c r="C719">
-        <v>39.493359269999999</v>
+        <v>39.49335927255094</v>
       </c>
       <c r="D719">
-        <v>15.89170043</v>
+        <v>15.89170042707072</v>
       </c>
     </row>
     <row r="720" spans="2:4">
@@ -15386,10 +15386,10 @@
         <v>1007</v>
       </c>
       <c r="C720">
-        <v>39.943019450000001</v>
+        <v>39.943019454413211</v>
       </c>
       <c r="D720">
-        <v>15.89170043</v>
+        <v>15.89170042707072</v>
       </c>
     </row>
     <row r="721" spans="2:4">
@@ -15397,10 +15397,10 @@
         <v>1008</v>
       </c>
       <c r="C721">
-        <v>40.392679639999997</v>
+        <v>40.392679636275481</v>
       </c>
       <c r="D721">
-        <v>15.89170043</v>
+        <v>15.89170042707072</v>
       </c>
     </row>
     <row r="722" spans="2:4">
@@ -15408,10 +15408,10 @@
         <v>1009</v>
       </c>
       <c r="C722">
-        <v>40.842339819999999</v>
+        <v>40.842339818137752</v>
       </c>
       <c r="D722">
-        <v>15.89170043</v>
+        <v>15.89170042707072</v>
       </c>
     </row>
     <row r="723" spans="2:4">
@@ -15419,10 +15419,10 @@
         <v>1010</v>
       </c>
       <c r="C723">
-        <v>41.292000000000002</v>
+        <v>41.292000000000016</v>
       </c>
       <c r="D723">
-        <v>15.89170043</v>
+        <v>15.89170042707072</v>
       </c>
     </row>
     <row r="724" spans="2:4">
@@ -15430,10 +15430,10 @@
         <v>1011</v>
       </c>
       <c r="C724">
-        <v>41.741660179999997</v>
+        <v>41.741660181862287</v>
       </c>
       <c r="D724">
-        <v>15.89170043</v>
+        <v>15.89170042707072</v>
       </c>
     </row>
     <row r="725" spans="2:4">
@@ -15441,10 +15441,10 @@
         <v>1012</v>
       </c>
       <c r="C725">
-        <v>42.191320359999999</v>
+        <v>42.191320363724557</v>
       </c>
       <c r="D725">
-        <v>15.89170043</v>
+        <v>15.89170042707072</v>
       </c>
     </row>
     <row r="726" spans="2:4">
@@ -15452,10 +15452,10 @@
         <v>1013</v>
       </c>
       <c r="C726">
-        <v>38.14437873</v>
+        <v>38.144378726964128</v>
       </c>
       <c r="D726">
-        <v>16.444317160000001</v>
+        <v>16.444317164915841</v>
       </c>
     </row>
     <row r="727" spans="2:4">
@@ -15463,10 +15463,10 @@
         <v>1014</v>
       </c>
       <c r="C727">
-        <v>38.594038910000002</v>
+        <v>38.594038908826398</v>
       </c>
       <c r="D727">
-        <v>16.444317160000001</v>
+        <v>16.444317164915841</v>
       </c>
     </row>
     <row r="728" spans="2:4">
@@ -15474,10 +15474,10 @@
         <v>1015</v>
       </c>
       <c r="C728">
-        <v>39.043699089999997</v>
+        <v>39.043699090688662</v>
       </c>
       <c r="D728">
-        <v>16.444317160000001</v>
+        <v>16.444317164915841</v>
       </c>
     </row>
     <row r="729" spans="2:4">
@@ -15485,10 +15485,10 @@
         <v>1016</v>
       </c>
       <c r="C729">
-        <v>39.493359269999999</v>
+        <v>39.49335927255094</v>
       </c>
       <c r="D729">
-        <v>16.444317160000001</v>
+        <v>16.444317164915841</v>
       </c>
     </row>
     <row r="730" spans="2:4">
@@ -15496,10 +15496,10 @@
         <v>1017</v>
       </c>
       <c r="C730">
-        <v>39.943019450000001</v>
+        <v>39.943019454413196</v>
       </c>
       <c r="D730">
-        <v>16.444317160000001</v>
+        <v>16.444317164915841</v>
       </c>
     </row>
     <row r="731" spans="2:4">
@@ -15507,10 +15507,10 @@
         <v>1018</v>
       </c>
       <c r="C731">
-        <v>40.392679639999997</v>
+        <v>40.392679636275481</v>
       </c>
       <c r="D731">
-        <v>16.444317160000001</v>
+        <v>16.444317164915841</v>
       </c>
     </row>
     <row r="732" spans="2:4">
@@ -15518,10 +15518,10 @@
         <v>1019</v>
       </c>
       <c r="C732">
-        <v>40.842339819999999</v>
+        <v>40.842339818137752</v>
       </c>
       <c r="D732">
-        <v>16.444317160000001</v>
+        <v>16.444317164915841</v>
       </c>
     </row>
     <row r="733" spans="2:4">
@@ -15529,10 +15529,10 @@
         <v>1020</v>
       </c>
       <c r="C733">
-        <v>41.292000000000002</v>
+        <v>41.292000000000023</v>
       </c>
       <c r="D733">
-        <v>16.444317160000001</v>
+        <v>16.444317164915841</v>
       </c>
     </row>
     <row r="734" spans="2:4">
@@ -15540,10 +15540,10 @@
         <v>1021</v>
       </c>
       <c r="C734">
-        <v>41.741660179999997</v>
+        <v>41.741660181862287</v>
       </c>
       <c r="D734">
-        <v>16.444317160000001</v>
+        <v>16.444317164915841</v>
       </c>
     </row>
     <row r="735" spans="2:4">
@@ -15551,10 +15551,10 @@
         <v>1022</v>
       </c>
       <c r="C735">
-        <v>39.043699089999997</v>
+        <v>39.043699090688662</v>
       </c>
       <c r="D735">
-        <v>16.996933899999998</v>
+        <v>16.996933902760961</v>
       </c>
     </row>
     <row r="736" spans="2:4">
@@ -15562,10 +15562,10 @@
         <v>1023</v>
       </c>
       <c r="C736">
-        <v>39.493359269999999</v>
+        <v>39.49335927255094</v>
       </c>
       <c r="D736">
-        <v>16.996933899999998</v>
+        <v>16.996933902760961</v>
       </c>
     </row>
     <row r="737" spans="2:4">
@@ -15573,10 +15573,10 @@
         <v>1024</v>
       </c>
       <c r="C737">
-        <v>40.392679639999997</v>
+        <v>40.392679636275481</v>
       </c>
       <c r="D737">
-        <v>16.996933899999998</v>
+        <v>16.996933902760961</v>
       </c>
     </row>
     <row r="738" spans="2:4">
@@ -15584,10 +15584,10 @@
         <v>1025</v>
       </c>
       <c r="C738">
-        <v>40.842339819999999</v>
+        <v>40.842339818137752</v>
       </c>
       <c r="D738">
-        <v>16.996933899999998</v>
+        <v>16.996933902760961</v>
       </c>
     </row>
     <row r="739" spans="2:4">
@@ -15595,10 +15595,10 @@
         <v>1026</v>
       </c>
       <c r="C739">
-        <v>41.292000000000002</v>
+        <v>41.292000000000023</v>
       </c>
       <c r="D739">
-        <v>16.996933899999998</v>
+        <v>16.996933902760961</v>
       </c>
     </row>
     <row r="740" spans="2:4">
@@ -15606,10 +15606,10 @@
         <v>1027</v>
       </c>
       <c r="C740">
-        <v>40.392679639999997</v>
+        <v>40.392679636275481</v>
       </c>
       <c r="D740">
-        <v>17.54955064</v>
+        <v>17.549550640606085</v>
       </c>
     </row>
     <row r="741" spans="2:4">
@@ -15617,10 +15617,10 @@
         <v>1028</v>
       </c>
       <c r="C741">
-        <v>40.842339819999999</v>
+        <v>40.842339818137752</v>
       </c>
       <c r="D741">
-        <v>17.54955064</v>
+        <v>17.549550640606085</v>
       </c>
     </row>
     <row r="742" spans="2:4">
@@ -15628,10 +15628,10 @@
         <v>1029</v>
       </c>
       <c r="C742">
-        <v>39.943019450000001</v>
+        <v>39.943019454413196</v>
       </c>
       <c r="D742">
-        <v>18.102167380000001</v>
+        <v>18.102167378451199</v>
       </c>
     </row>
     <row r="743" spans="2:4">
@@ -15639,10 +15639,10 @@
         <v>1030</v>
       </c>
       <c r="C743">
-        <v>40.392679639999997</v>
+        <v>40.392679636275481</v>
       </c>
       <c r="D743">
-        <v>18.102167380000001</v>
+        <v>18.102167378451199</v>
       </c>
     </row>
     <row r="744" spans="2:4">
@@ -15650,10 +15650,10 @@
         <v>1031</v>
       </c>
       <c r="C744">
-        <v>40.842339819999999</v>
+        <v>40.842339818137752</v>
       </c>
       <c r="D744">
-        <v>18.102167380000001</v>
+        <v>18.102167378451199</v>
       </c>
     </row>
     <row r="745" spans="2:4">
@@ -17983,7 +17983,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E38EFBB-F980-4CE9-8E40-838D5D71BDD8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA5C097F-B768-4FF2-9D22-10020B0B02C3}">
   <dimension ref="B2:D948"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-09 00:05
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D15C424E-D252-4728-850A-CDF33126D3CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E894CFD1-9616-4060-840D-383372CC5FEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9912,7 +9912,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F9C3722-0659-44DE-AC83-BE6F4C08D861}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B59AC1F-370E-4304-A60A-71CC77E7132C}">
   <dimension ref="B9:D955"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -20333,7 +20333,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{633A268D-5D22-4714-9B3C-C936B72017BF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E092F9AE-90A8-453C-AF31-3D1E4DB01A33}">
   <dimension ref="B2:D948"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-11 19:48
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1C28C6C-706B-48E9-AD03-E6F0FFA44890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{810A17DB-895B-4D3E-B344-F88E844F0198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B921BD27-E104-432A-AB35-3389DFB47981}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F64AF3B-A85C-4F1E-9A31-9B16EFD382BC}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25123D52-84D0-4CB5-9920-6B91DAEBF070}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{983C5538-7B8D-4ED0-B15E-BF5B0313C0DA}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-12 13:31
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{810A17DB-895B-4D3E-B344-F88E844F0198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{53C92933-51F4-43A9-AF65-5A819C158232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F64AF3B-A85C-4F1E-9A31-9B16EFD382BC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26B40ACA-BAF1-43D8-ADA0-D7B42C1F63E6}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{983C5538-7B8D-4ED0-B15E-BF5B0313C0DA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBCFBECB-CF4F-455B-8112-E19E4E5D9883}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-13 10:48
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{53C92933-51F4-43A9-AF65-5A819C158232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{69604435-6385-4B95-B042-2C3FEF60077F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26B40ACA-BAF1-43D8-ADA0-D7B42C1F63E6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C78499A1-4F35-4E19-A0A2-376C75E1DCA3}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBCFBECB-CF4F-455B-8112-E19E4E5D9883}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FDDBCBA-5346-46E4-BB5E-253F3C575A4E}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-13 12:02
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{69604435-6385-4B95-B042-2C3FEF60077F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{84D795C2-00F8-43EE-8730-4E385A03E5EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C78499A1-4F35-4E19-A0A2-376C75E1DCA3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B1BA48F-129D-4F4E-92DF-B886D20BF74F}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FDDBCBA-5346-46E4-BB5E-253F3C575A4E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{134E586F-20B5-4FCF-97C6-8B6C8F744E45}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-13 14:08
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{84D795C2-00F8-43EE-8730-4E385A03E5EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A999603-FBBB-478F-B904-F5D09D02B2A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B1BA48F-129D-4F4E-92DF-B886D20BF74F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33877C04-BED0-459D-90FC-66A3D2965057}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{134E586F-20B5-4FCF-97C6-8B6C8F744E45}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A7A7393-2C98-48C8-AC37-62B859391223}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-13 14:52
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A999603-FBBB-478F-B904-F5D09D02B2A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{092E001B-4021-4C6C-A69F-3D4AAF8EA983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33877C04-BED0-459D-90FC-66A3D2965057}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B7091F6-F612-4074-A4D5-8AB410797C40}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A7A7393-2C98-48C8-AC37-62B859391223}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B7EF03F-C40A-4ED1-872D-B101E06AA0B7}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-13 15:25
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{092E001B-4021-4C6C-A69F-3D4AAF8EA983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8E4EFB9E-1025-4A1B-82B4-923863D8BB3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B7091F6-F612-4074-A4D5-8AB410797C40}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1512D35F-0E40-4D12-B0F7-F3AC9826E8FB}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B7EF03F-C40A-4ED1-872D-B101E06AA0B7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F36988A-AE84-4DD7-909E-177A8CACF426}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-13 16:00
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8E4EFB9E-1025-4A1B-82B4-923863D8BB3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E024DC2B-2120-4CED-9C79-4EBF371AF94C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1512D35F-0E40-4D12-B0F7-F3AC9826E8FB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{000A0FFC-1955-44DB-83F7-8E73926D895D}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F36988A-AE84-4DD7-909E-177A8CACF426}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{695A0DDD-3781-4234-BD08-CFF7EB3B7F13}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-13 17:35
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E024DC2B-2120-4CED-9C79-4EBF371AF94C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1231FD3F-60C2-4BC7-A770-DD7ADEB219AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{000A0FFC-1955-44DB-83F7-8E73926D895D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D32C2C6A-F80F-405D-8F90-313B6DC3B9B3}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{695A0DDD-3781-4234-BD08-CFF7EB3B7F13}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8CFF938-D637-44A1-9F26-726CC8790F93}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-14 20:05
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1231FD3F-60C2-4BC7-A770-DD7ADEB219AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C667203F-23B0-44A5-850D-9A20CB7A1976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D32C2C6A-F80F-405D-8F90-313B6DC3B9B3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{457699D6-2D31-4E52-81C8-55129DBA7954}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8CFF938-D637-44A1-9F26-726CC8790F93}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F60053EB-51C6-4D83-A9AB-BE2F94A91E84}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-15 00:03
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C667203F-23B0-44A5-850D-9A20CB7A1976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{74940815-FDF0-4192-97B0-E4CA5EB15EA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{457699D6-2D31-4E52-81C8-55129DBA7954}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9F22DC8-27C1-4C38-BF41-13F34AB0A638}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F60053EB-51C6-4D83-A9AB-BE2F94A91E84}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A66A0E2-E619-4A3C-96AA-132C91378803}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-15 00:15
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{74940815-FDF0-4192-97B0-E4CA5EB15EA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C040624-34CF-49CB-8A58-20740F03B74D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9F22DC8-27C1-4C38-BF41-13F34AB0A638}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B1A6AE3-04CC-41B0-BE0D-8F8B89CBDA8E}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A66A0E2-E619-4A3C-96AA-132C91378803}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63A78A55-766E-4306-8B62-CA61DE6311EF}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-15 00:24
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C040624-34CF-49CB-8A58-20740F03B74D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E4F1396-A584-4705-9EA8-63F444DF6CD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B1A6AE3-04CC-41B0-BE0D-8F8B89CBDA8E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3C4E93B-2972-4F64-875D-30CF75FCF271}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63A78A55-766E-4306-8B62-CA61DE6311EF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0BF9D70-081B-44A8-B37F-6B4AA5CF8E64}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-15 00:29
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E4F1396-A584-4705-9EA8-63F444DF6CD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1520953-5051-4987-8129-F44C0BD0CE45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3C4E93B-2972-4F64-875D-30CF75FCF271}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A0D7F65-2990-4064-9B93-5627FBA84A53}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0BF9D70-081B-44A8-B37F-6B4AA5CF8E64}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96982F80-9425-4B4B-B2E0-D78DC8888BAD}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-15 00:33
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1520953-5051-4987-8129-F44C0BD0CE45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{713D8CF6-C590-4FBA-B583-4EF5B47D170A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1241,13 +1241,13 @@
     <t>g64</t>
   </si>
   <si>
-    <t>f97p50</t>
-  </si>
-  <si>
     <t>f96p10</t>
   </si>
   <si>
     <t>f96p90</t>
+  </si>
+  <si>
+    <t>f96p50</t>
   </si>
   <si>
     <t>grid_node</t>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A0D7F65-2990-4064-9B93-5627FBA84A53}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AE64871-9693-43B8-A74D-DB83DA6AF636}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96982F80-9425-4B4B-B2E0-D78DC8888BAD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12C93B49-68BD-4A4A-8248-EF3E63B9265E}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28594,7 +28594,7 @@
         <v>337</v>
       </c>
       <c r="U12" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="13" spans="2:24">
@@ -28637,7 +28637,7 @@
         <v>343</v>
       </c>
       <c r="U13" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="14" spans="2:24">
@@ -28680,7 +28680,7 @@
         <v>349</v>
       </c>
       <c r="U14" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="15" spans="2:24">
@@ -29497,11 +29497,11 @@
       </c>
       <c r="C36" t="str">
         <f t="shared" si="5"/>
-        <v>e 1.5 deg no OS.f97p50</v>
+        <v>e 1.5 deg no OS.f96p50</v>
       </c>
       <c r="H36" t="str">
         <f t="shared" si="2"/>
-        <v>e 1.5 deg no OS.f97p50</v>
+        <v>e 1.5 deg no OS.f96p50</v>
       </c>
       <c r="I36" t="str">
         <f t="shared" si="3"/>
@@ -29509,7 +29509,7 @@
       </c>
       <c r="J36" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N36">
         <v>5</v>
@@ -29534,11 +29534,11 @@
       </c>
       <c r="C37" t="str">
         <f t="shared" si="5"/>
-        <v>d 1.5 deg OS.f97p50</v>
+        <v>d 1.5 deg OS.f96p50</v>
       </c>
       <c r="H37" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.f97p50</v>
+        <v>d 1.5 deg OS.f96p50</v>
       </c>
       <c r="I37" t="str">
         <f t="shared" si="3"/>
@@ -29546,7 +29546,7 @@
       </c>
       <c r="J37" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N37">
         <v>5</v>
@@ -29571,11 +29571,11 @@
       </c>
       <c r="C38" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).f97p50</v>
+        <v>c 2 deg (67%).f96p50</v>
       </c>
       <c r="H38" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).f97p50</v>
+        <v>c 2 deg (67%).f96p50</v>
       </c>
       <c r="I38" t="str">
         <f t="shared" si="3"/>
@@ -29583,7 +29583,7 @@
       </c>
       <c r="J38" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N38">
         <v>5</v>
@@ -29608,11 +29608,11 @@
       </c>
       <c r="C39" t="str">
         <f t="shared" si="5"/>
-        <v>b 2 deg (50%).f97p50</v>
+        <v>b 2 deg (50%).f96p50</v>
       </c>
       <c r="H39" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).f97p50</v>
+        <v>b 2 deg (50%).f96p50</v>
       </c>
       <c r="I39" t="str">
         <f t="shared" si="3"/>
@@ -29620,7 +29620,7 @@
       </c>
       <c r="J39" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N39">
         <v>5</v>
@@ -29645,11 +29645,11 @@
       </c>
       <c r="C40" t="str">
         <f t="shared" si="5"/>
-        <v>a 3 deg.f97p50</v>
+        <v>a 3 deg.f96p50</v>
       </c>
       <c r="H40" t="str">
         <f t="shared" si="2"/>
-        <v>a 3 deg.f97p50</v>
+        <v>a 3 deg.f96p50</v>
       </c>
       <c r="I40" t="str">
         <f t="shared" si="3"/>
@@ -29657,7 +29657,7 @@
       </c>
       <c r="J40" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N40">
         <v>5</v>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-15 00:52
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{713D8CF6-C590-4FBA-B583-4EF5B47D170A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BBEFB599-5D7F-47ED-880A-E8BFEC8AC370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AE64871-9693-43B8-A74D-DB83DA6AF636}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{653A8EBE-B3C2-45FF-BAA2-022ED0DC4022}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12C93B49-68BD-4A4A-8248-EF3E63B9265E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54420672-0849-4D0F-B707-EAAA1412D09F}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-16 23:37
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BBEFB599-5D7F-47ED-880A-E8BFEC8AC370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C6085C1-0218-4A78-92A3-394CB5A19E22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1103" yWindow="1103" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{653A8EBE-B3C2-45FF-BAA2-022ED0DC4022}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AD44E60-3973-4A0F-8248-D36C167239BF}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54420672-0849-4D0F-B707-EAAA1412D09F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AF326E4-334A-4D60-8ABC-4F901D580365}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-17 01:08
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C6085C1-0218-4A78-92A3-394CB5A19E22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0432CBDA-7561-45FF-A8E1-B375A39509BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1103" yWindow="1103" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2573" yWindow="2573" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AD44E60-3973-4A0F-8248-D36C167239BF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BF364EF-2073-4D09-911F-40994277FE87}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AF326E4-334A-4D60-8ABC-4F901D580365}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E935741E-78B8-434B-9CF2-FE02F164665D}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-17 01:15
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0432CBDA-7561-45FF-A8E1-B375A39509BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F560D43D-8B2C-4670-8EF2-86E1CC24726B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2573" yWindow="2573" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3308" yWindow="3308" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BF364EF-2073-4D09-911F-40994277FE87}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FE5DEBE-1585-42DC-8F1F-49A073CB3CE7}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E935741E-78B8-434B-9CF2-FE02F164665D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35C6BCF1-5C05-47CA-BC64-8BCD0DA9EEC0}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-17 02:03
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F560D43D-8B2C-4670-8EF2-86E1CC24726B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{97EEC93D-9F27-4BE0-B687-E033968531BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3308" yWindow="3308" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FE5DEBE-1585-42DC-8F1F-49A073CB3CE7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C676A9B-C773-46CD-A619-4CB01F8EF4A5}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35C6BCF1-5C05-47CA-BC64-8BCD0DA9EEC0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3FBF90A-3BAF-4411-A610-30D69218F516}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-17 09:35
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97EEC93D-9F27-4BE0-B687-E033968531BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4DD3F641-4802-4CD1-A683-8517AC3BCE8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3308" yWindow="3308" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C676A9B-C773-46CD-A619-4CB01F8EF4A5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{582E371B-CFF0-4EFD-8F47-E21A5FBE24C3}">
   <dimension ref="B9:D688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14563,7 +14563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3FBF90A-3BAF-4411-A610-30D69218F516}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0FACC57-95F8-4D87-90A0-38E7C902C288}">
   <dimension ref="B9:H688"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-19 18:23
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7AF1D803-BA6F-4103-B5C9-E7C7C85C56A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A467734-F460-486C-AF02-7B4F9BE4E836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8882,7 +8882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FEFD558-E1B3-4D68-901C-EB075401B146}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B96AD11-FF13-4FA6-9991-6175C3FB2460}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12439,7 +12439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6371F6B-CDD8-4C59-8E8F-FA148050C986}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7BF8833-74B3-4BB7-8507-1A598C77A1D9}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-19 19:27
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A467734-F460-486C-AF02-7B4F9BE4E836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{91641DB4-0A72-4E19-97E2-3C71162388A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8882,7 +8882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B96AD11-FF13-4FA6-9991-6175C3FB2460}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A50A8F9-C4CF-4DDB-895B-5CC4D16FF906}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12439,7 +12439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7BF8833-74B3-4BB7-8507-1A598C77A1D9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC68BD4E-4634-40D2-9A84-7FCF7E8E3CB2}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-19 19:33
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{91641DB4-0A72-4E19-97E2-3C71162388A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{932E81CE-53D6-4F4E-A2A8-EB21F7544555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8882,7 +8882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A50A8F9-C4CF-4DDB-895B-5CC4D16FF906}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A59972C-F511-49BC-9827-3F05227FDA3C}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12439,7 +12439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC68BD4E-4634-40D2-9A84-7FCF7E8E3CB2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A937174-A24E-4846-B30C-4C973923BA9D}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-19 19:37
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{932E81CE-53D6-4F4E-A2A8-EB21F7544555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F078F00-A0EE-46FB-8F9D-47768DC85B75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8882,7 +8882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A59972C-F511-49BC-9827-3F05227FDA3C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F265C2F-2D61-4211-805F-144DF4F375D6}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12439,7 +12439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A937174-A24E-4846-B30C-4C973923BA9D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80762CCF-15A1-4186-8723-787C2FBF3308}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-19 19:42
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F078F00-A0EE-46FB-8F9D-47768DC85B75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{916A79B0-8767-4222-96FF-7CB61768858A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8882,7 +8882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F265C2F-2D61-4211-805F-144DF4F375D6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0810C8A5-DF2A-4628-9E88-244BD0DF2C7D}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12439,7 +12439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80762CCF-15A1-4186-8723-787C2FBF3308}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3A67EDE-E25A-4A5B-BDD5-F24ACBD85935}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-19 19:47
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{916A79B0-8767-4222-96FF-7CB61768858A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{79DAB187-3173-43B8-8FA0-E8CA4E1C4097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8882,7 +8882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0810C8A5-DF2A-4628-9E88-244BD0DF2C7D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{187B6D67-7C10-4AA3-A7D7-A5E96934ED06}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12439,7 +12439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3A67EDE-E25A-4A5B-BDD5-F24ACBD85935}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DDB0BD1-AE35-47D2-906E-482CF69EFD21}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-19 19:52
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{79DAB187-3173-43B8-8FA0-E8CA4E1C4097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C30D3AD1-8617-42C2-9C1E-C3665B4210B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8882,7 +8882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{187B6D67-7C10-4AA3-A7D7-A5E96934ED06}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FA484ED-E9CA-4A7F-AC32-0F93FC240CF1}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12439,7 +12439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DDB0BD1-AE35-47D2-906E-482CF69EFD21}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B47DE18-059C-4F12-B19B-B13A3B14F656}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-19 19:56
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C30D3AD1-8617-42C2-9C1E-C3665B4210B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B6592C0-4702-447B-A2A6-2D5878541563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8882,7 +8882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FA484ED-E9CA-4A7F-AC32-0F93FC240CF1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CB6F1F1-CEA3-4452-AADF-DB095BBA17C4}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12439,7 +12439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B47DE18-059C-4F12-B19B-B13A3B14F656}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB5A2AC6-64D0-469A-AA60-44888BFB5A64}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-19 20:02
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B6592C0-4702-447B-A2A6-2D5878541563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{69AEC4DE-F777-48A3-AD8D-35DB770D80C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8882,7 +8882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CB6F1F1-CEA3-4452-AADF-DB095BBA17C4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4AD2CFE-81FB-49E6-A33C-CE8886F66CD8}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12439,7 +12439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB5A2AC6-64D0-469A-AA60-44888BFB5A64}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D77027F4-6533-4E59-BF67-A60BE4CB2BF0}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-19 20:09
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{69AEC4DE-F777-48A3-AD8D-35DB770D80C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2726594A-081F-45E9-AFFE-AAFA0AA52A82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8882,7 +8882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4AD2CFE-81FB-49E6-A33C-CE8886F66CD8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2309FB11-E973-403B-AC32-FA42988AECB0}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12439,7 +12439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D77027F4-6533-4E59-BF67-A60BE4CB2BF0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7056C2C-046C-4B78-89A2-23CEA1109765}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-19 20:12
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2726594A-081F-45E9-AFFE-AAFA0AA52A82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A3C7E938-C68C-4480-B7C8-80A82260BF8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8882,7 +8882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2309FB11-E973-403B-AC32-FA42988AECB0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0D36012-EBEA-440E-83BE-07D01E32B67B}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12439,7 +12439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7056C2C-046C-4B78-89A2-23CEA1109765}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C3680E9-5268-418E-B7C2-BDBA07864B79}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-19 20:28
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A3C7E938-C68C-4480-B7C8-80A82260BF8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6CE9123-EBDA-430C-AD02-FAF744A6B2A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8882,7 +8882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0D36012-EBEA-440E-83BE-07D01E32B67B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A489E09-E1F6-46E2-8454-C0DEF1329DE9}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12439,7 +12439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C3680E9-5268-418E-B7C2-BDBA07864B79}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93D8DA96-2EB8-4FC8-81AA-A8BACEC7A068}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-19 23:00
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6CE9123-EBDA-430C-AD02-FAF744A6B2A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{35ADE424-45BD-4E9C-A58E-5E33FBD04F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8882,7 +8882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A489E09-E1F6-46E2-8454-C0DEF1329DE9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB566D71-FD0B-48FF-BA9C-A596D7B18471}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12439,7 +12439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93D8DA96-2EB8-4FC8-81AA-A8BACEC7A068}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F94E1F7F-64A0-41FC-83E0-BDA7F13D5008}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-20 08:52
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{35ADE424-45BD-4E9C-A58E-5E33FBD04F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{00485834-B424-4762-A01D-6E3C46A65035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8882,7 +8882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB566D71-FD0B-48FF-BA9C-A596D7B18471}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E28E92A6-7B23-4B8E-A447-094AAB58431E}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12439,7 +12439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F94E1F7F-64A0-41FC-83E0-BDA7F13D5008}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB6D5CB7-34A4-4F93-B5DE-27A27B9A4638}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-20 08:59
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{00485834-B424-4762-A01D-6E3C46A65035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AD50563B-9A6E-4E75-83CC-C1F05895161D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8882,7 +8882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E28E92A6-7B23-4B8E-A447-094AAB58431E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C81DAF3F-A961-439E-9B9B-EC2DB8246524}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12439,7 +12439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB6D5CB7-34A4-4F93-B5DE-27A27B9A4638}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BA379B7-802A-4CCA-98AB-B75243B2F645}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-22 03:18
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{28ED0389-912F-457A-86D0-C2778D72FD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5EF590B2-BB1F-4F81-8D6D-BE5F08A09881}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8897,7 +8897,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD48F1B9-BA80-4EC5-B360-D502A8B96E93}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24114CD2-BB59-400E-BC7B-360C61C1EDE4}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12112,10 +12112,10 @@
         <v>695</v>
       </c>
       <c r="C301">
-        <v>43.090640727449113</v>
+        <v>44.21479118210479</v>
       </c>
       <c r="D301">
-        <v>13.865439054971944</v>
+        <v>12.668102789640848</v>
       </c>
     </row>
     <row r="302" spans="2:4">
@@ -12123,10 +12123,10 @@
         <v>696</v>
       </c>
       <c r="C302">
-        <v>44.21479118210479</v>
+        <v>41.966490272793422</v>
       </c>
       <c r="D302">
-        <v>12.668102789640848</v>
+        <v>15.062775320303036</v>
       </c>
     </row>
     <row r="303" spans="2:4">
@@ -12134,10 +12134,10 @@
         <v>697</v>
       </c>
       <c r="C303">
-        <v>41.966490272793422</v>
+        <v>43.090640727449113</v>
       </c>
       <c r="D303">
-        <v>15.062775320303036</v>
+        <v>13.865439054971944</v>
       </c>
     </row>
     <row r="304" spans="2:4">
@@ -12145,10 +12145,10 @@
         <v>698</v>
       </c>
       <c r="C304">
-        <v>40.683636224539292</v>
+        <v>40.632498399935351</v>
       </c>
       <c r="D304">
-        <v>16.931920168896827</v>
+        <v>17.070616134473646</v>
       </c>
     </row>
     <row r="305" spans="2:4">
@@ -12156,10 +12156,10 @@
         <v>699</v>
       </c>
       <c r="C305">
-        <v>40.842339818137752</v>
+        <v>40.906576986975217</v>
       </c>
       <c r="D305">
-        <v>15.339083689225598</v>
+        <v>15.496974185752777</v>
       </c>
     </row>
     <row r="306" spans="2:4">
@@ -12420,10 +12420,10 @@
         <v>723</v>
       </c>
       <c r="C329">
-        <v>36.425471789132992</v>
+        <v>36.356293299615722</v>
       </c>
       <c r="D329">
-        <v>14.726193410011531</v>
+        <v>14.824868933948331</v>
       </c>
     </row>
     <row r="330" spans="2:4">
@@ -12431,10 +12431,10 @@
         <v>724</v>
       </c>
       <c r="C330">
-        <v>35.681803026822308</v>
+        <v>37.435477736085161</v>
       </c>
       <c r="D330">
-        <v>12.717441672726681</v>
+        <v>12.882370762735327</v>
       </c>
     </row>
     <row r="331" spans="2:4">
@@ -12442,10 +12442,10 @@
         <v>725</v>
       </c>
       <c r="C331">
-        <v>36.940851536036668</v>
+        <v>36.067226039847121</v>
       </c>
       <c r="D331">
-        <v>12.552512582718029</v>
+        <v>12.599635179863361</v>
       </c>
     </row>
   </sheetData>
@@ -12454,7 +12454,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70156052-1586-4EC5-81F6-4B5F20B0790D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4310024-CA72-46BB-A0CE-26A231243813}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-22 11:23
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5EF590B2-BB1F-4F81-8D6D-BE5F08A09881}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{13229BE9-4CEB-4AB4-9748-D8A8E7F3AB7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8897,7 +8897,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24114CD2-BB59-400E-BC7B-360C61C1EDE4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36602722-CD50-4C54-A403-4C703B277BE6}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12454,7 +12454,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4310024-CA72-46BB-A0CE-26A231243813}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12B7645A-31CC-4EF6-A8C4-A4DFA928E7B3}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-22 11:56
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{13229BE9-4CEB-4AB4-9748-D8A8E7F3AB7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5887FD2F-8E1D-4FE5-B331-EDCA2106AB07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8897,7 +8897,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36602722-CD50-4C54-A403-4C703B277BE6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEFB282F-5073-4B37-B0AC-8C41F5DF4F24}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12454,7 +12454,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12B7645A-31CC-4EF6-A8C4-A4DFA928E7B3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C2B441F-1E62-42A9-A32F-C0F104AC70C6}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-22 13:10
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5887FD2F-8E1D-4FE5-B331-EDCA2106AB07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F1F938D-E962-4B7B-9A4E-7B4D86482132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8897,7 +8897,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEFB282F-5073-4B37-B0AC-8C41F5DF4F24}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB92A5DF-6D77-4FB3-8247-93D22F4B5198}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12454,7 +12454,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C2B441F-1E62-42A9-A32F-C0F104AC70C6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53518DBE-0A14-42DB-8360-129B4FE2B18C}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-22 14:02
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F1F938D-E962-4B7B-9A4E-7B4D86482132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3F6CEEC4-4D9F-4A82-BCA9-87654454C1EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8897,7 +8897,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB92A5DF-6D77-4FB3-8247-93D22F4B5198}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6864EA2-A8B9-4187-A227-6EF965154A57}">
   <dimension ref="B9:D331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12454,7 +12454,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53518DBE-0A14-42DB-8360-129B4FE2B18C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A3998A2-AE98-4FA8-A046-5B4228A476D5}">
   <dimension ref="B9:H331"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-27 20:40
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F2552027-5ECB-45AC-9457-37CC79108EBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6804D8BB-6A4F-438F-A6AA-16F8689D52C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10993,7 +10993,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C30EE91-4127-4323-B4D7-6DE220E668A3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A8EF5AC-8C19-4797-A448-0E2E2DF0F7F3}">
   <dimension ref="B9:H337"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -17517,7 +17517,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E62A3CEC-B0B0-4DD1-8283-38F59AC67F69}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C761C054-256C-4E9C-97CC-257EA1F452F6}">
   <dimension ref="B9:L337"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>